<commit_message>
Add predictions batch 2026-07-26 to history/
</commit_message>
<xml_diff>
--- a/history/2026-07-26/VIP_2026-07-26.xlsx
+++ b/history/2026-07-26/VIP_2026-07-26.xlsx
@@ -137,8 +137,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PredTable" displayName="PredTable" ref="A1:O41" headerRowCount="1">
-  <autoFilter ref="A1:O41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PredTable" displayName="PredTable" ref="A1:O47" headerRowCount="1">
+  <autoFilter ref="A1:O47"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Division"/>
     <tableColumn id="2" name="Date"/>
@@ -449,13 +449,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -924,7 +924,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>SE Allsvenskan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -934,62 +934,62 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>20:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Sirius</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Botafogo RJ</t>
+          <t>Goteborg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home Win</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>89.00%</t>
+          <t>93.00%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>OOUOOU</t>
+          <t>WWWWWD</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>OOOUUO</t>
+          <t>DDLWWL</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. Botafogo RJ concedes 1.9 goals at away. Both sides look capable of goals.</t>
+          <t>Sirius has won 5 of their last 6 home games. Goteborg has won 2 of their last 6 home games. Goteborg concedes 2.9 goals at away. Strong home record supports this.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
+          <t>13M 11W 2D 0L 36-16 (2.8-1.2) | Home: 6M 5W 1D 0L 17-8 (2.8-1.3)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
+          <t>13M 3W 4D 6L 16-29 (1.2-2.2) | Away: 7M 2W 2D 3L 10-20 (1.4-2.9)</t>
         </is>
       </c>
       <c r="O7" t="b">
@@ -999,7 +999,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CH Super League</t>
+          <t>BR Serie A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1009,17 +1009,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Young Boys</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sion</t>
+          <t>Botafogo RJ</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1034,37 +1034,37 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>85.00%</t>
+          <t>89.00%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>8/8</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>OUUOOO</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>OOOUOO</t>
+          <t>OOOUUO</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Young Boys averages 2.3 goals at home. Sion averages 1.8 goals at away. Young Boys concedes 1.3 goals at home. Sion concedes 1.4 goals at away. Both sides look capable of goals.</t>
+          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. Botafogo RJ concedes 1.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>38M 15W 10D 13L 80-69 (2.1-1.8) | Home: 19M 9W 5D 5L 43-25 (2.3-1.3)</t>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>38M 16W 15D 7L 63-40 (1.7-1.1) | Away: 19M 7W 8D 4L 34-26 (1.8-1.4)</t>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
         </is>
       </c>
       <c r="O8" t="b">
@@ -1084,17 +1084,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sonderjyske</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Midtjylland</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1109,37 +1109,32 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>83.00%</t>
+          <t>86.00%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>UUUOOO</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>OUOOUU</t>
+          <t>OOOOOO</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Sonderjyske averages 1.6 goals at home. Midtjylland averages 1.8 goals at away. Sonderjyske concedes 1.2 goals at home. Midtjylland concedes 0.8 goals at away. Both sides look capable of goals.</t>
+          <t>FC Copenhagen averages 2.1 goals at home. Lyngby averages 0.0 goals at away. FC Copenhagen concedes 1.2 goals at home. Lyngby concedes 0.0 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>32M 12W 8D 12L 44-49 (1.4-1.5) | Home: 16M 8W 3D 5L 25-20 (1.6-1.2)</t>
+          <t>32M 15W 6D 11L 67-44 (2.1-1.4) | Home: 16M 7W 4D 5L 33-19 (2.1-1.2)</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>32M 16W 12D 4L 72-36 (2.2-1.1) | Away: 16M 8W 6D 2L 29-12 (1.8-0.8)</t>
+          <t>0M 0W 0D 0L 0-0 (0.0-0.0)</t>
         </is>
       </c>
       <c r="O9" t="b">
@@ -1149,7 +1144,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CH Super League</t>
+          <t>SE Allsvenskan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1159,22 +1154,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15:30:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>St. Gallen</t>
+          <t>Sirius</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Goteborg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home team Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1184,37 +1179,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>83.00%</t>
+          <t>86.00%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>9/10</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>OOUOOU</t>
+          <t>UOOUOO</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>OOOOOU</t>
+          <t>UUOOOO</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>St. Gallen averages 1.7 goals at home. Zurich averages 1.1 goals at away. St. Gallen concedes 1.2 goals at home. Zurich concedes 1.9 goals at away. Both sides look capable of goals.</t>
+          <t>Sirius averages 2.8 goals at home. Goteborg concedes 2.9 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>38M 20W 10D 8L 72-47 (1.9-1.2) | Home: 19M 10W 3D 6L 33-23 (1.7-1.2)</t>
+          <t>13M 11W 2D 0L 36-16 (2.8-1.2) | Home: 6M 5W 1D 0L 17-8 (2.8-1.3)</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>38M 11W 5D 22L 49-72 (1.3-1.9) | Away: 19M 4W 4D 11L 20-36 (1.1-1.9)</t>
+          <t>13M 3W 4D 6L 16-29 (1.2-2.2) | Away: 7M 2W 2D 3L 10-20 (1.4-2.9)</t>
         </is>
       </c>
       <c r="O10" t="b">
@@ -1224,7 +1219,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>CH Super League</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1234,22 +1229,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Young Boys</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Sion</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Home team Over 1.5 Goals</t>
+          <t>Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1259,37 +1254,37 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>83.00%</t>
+          <t>85.00%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>8/8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>OUOOOO</t>
+          <t>OUUOOO</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>UUOUUO</t>
+          <t>OOOUOO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Brann averages 1.5 goals at home. Valerenga concedes 2.2 goals at away. The home side’s attack should produce the required goals.</t>
+          <t>Young Boys averages 2.3 goals at home. Sion averages 1.8 goals at away. Young Boys concedes 1.3 goals at home. Sion concedes 1.4 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
+          <t>38M 15W 10D 13L 80-69 (2.1-1.8) | Home: 19M 9W 5D 5L 43-25 (2.3-1.3)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
+          <t>38M 16W 15D 7L 63-40 (1.7-1.1) | Away: 19M 7W 8D 4L 34-26 (1.8-1.4)</t>
         </is>
       </c>
       <c r="O11" t="b">
@@ -1309,22 +1304,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18:15:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Away team Over 1.5 Goals</t>
+          <t>Home team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1339,32 +1334,32 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>OOUOOO</t>
+          <t>OUOOOO</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>UOUOUO</t>
+          <t>UUOUUO</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. The away side’s attack looks likely to score well.</t>
+          <t>Brann averages 1.5 goals at home. Valerenga concedes 2.2 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O12" t="b">
@@ -1384,22 +1379,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Over 2.5 Goals</t>
+          <t>Away team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1409,37 +1404,37 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>82.00%</t>
+          <t>83.00%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>OUOOOO</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>UUOUUO</t>
+          <t>UOUOUO</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Brann concedes 1.3 goals at home. Valerenga concedes 2.2 goals at away. Both sides look capable of goals.</t>
+          <t>Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. The away side’s attack looks likely to score well.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O13" t="b">
@@ -1459,17 +1454,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>18:15:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1489,32 +1484,32 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>OOUOOO</t>
+          <t>OUOOOO</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>UOUOUO</t>
+          <t>UUOUUO</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. Viking concedes 0.9 goals at away. Both sides look capable of goals.</t>
+          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Brann concedes 1.3 goals at home. Valerenga concedes 2.2 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O14" t="b">
@@ -1524,7 +1519,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SE Allsvenskan</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1534,22 +1529,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>15:30:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Malmo FF</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Elfsborg</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1564,32 +1559,32 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>OOOOOO</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>OUOUOU</t>
+          <t>UOUOUO</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Malmo FF averages 3.0 goals at home. Elfsborg averages 1.2 goals at away. Malmo FF concedes 2.0 goals at home. Elfsborg concedes 1.3 goals at away. Both sides look capable of goals.</t>
+          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. Viking concedes 0.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>13M 6W 2D 5L 27-22 (2.1-1.7) | Home: 6M 3W 0D 3L 18-12 (3.0-2.0)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>14M 4W 6D 4L 18-17 (1.3-1.2) | Away: 6M 1W 3D 2L 7-8 (1.2-1.3)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O15" t="b">
@@ -1614,17 +1609,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Sirius</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Goteborg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Over 3.5 Goals</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1634,41 +1629,41 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>81.00%</t>
+          <t>82.00%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-OOUUO</t>
+          <t>UOOUOO</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>UUUUOO</t>
+          <t>UUOOOO</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Brommapojkarna averages 1.2 goals at home. Hammarby averages 1.0 goals at away. Brommapojkarna concedes 1.4 goals at home. Hammarby concedes 1.5 goals at away. Both sides look capable of goals.</t>
+          <t>Sirius averages 2.8 goals at home. Goteborg averages 1.4 goals at away. Sirius concedes 1.3 goals at home. Goteborg concedes 2.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>13M 4W 4D 5L 18-21 (1.4-1.6) | Home: 5M 1W 2D 2L 6-7 (1.2-1.4)</t>
+          <t>13M 11W 2D 0L 36-16 (2.8-1.2) | Home: 6M 5W 1D 0L 17-8 (2.8-1.3)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>14M 8W 2D 4L 32-14 (2.3-1.0) | Away: 6M 2W 1D 3L 6-9 (1.0-1.5)</t>
+          <t>13M 3W 4D 6L 16-29 (1.2-2.2) | Away: 7M 2W 2D 3L 10-20 (1.4-2.9)</t>
         </is>
       </c>
       <c r="O16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1684,62 +1679,62 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16:00:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sarpsborg 08</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HamKam</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home Win</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>78.00%</t>
+          <t>77.00%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>UUUOOU</t>
+          <t>LLWWLW</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>OUOOOO</t>
+          <t>WDLLLL</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Sarpsborg 08 averages 1.2 goals at home. HamKam averages 1.2 goals at away. Sarpsborg 08 concedes 0.8 goals at home. HamKam concedes 2.3 goals at away. Both sides look capable of goals.</t>
+          <t>Brann has won 3 of their last 6 home games. Valerenga has won 1 of their last 6 home games. Valerenga concedes 2.2 goals at away. Strong home record supports this.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>13M 5W 3D 5L 14-16 (1.1-1.2) | Home: 6M 3W 2D 1L 7-5 (1.2-0.8)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>13M 5W 3D 5L 20-25 (1.5-1.9) | Away: 6M 0W 3D 3L 7-14 (1.2-2.3)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O17" t="b">
@@ -1749,7 +1744,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AR Liga Profesional</t>
+          <t>SE Allsvenskan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1759,32 +1754,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>15:30:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Atl. Tucuman</t>
+          <t>GAIS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ind. Rivadavia</t>
+          <t>Halmstad</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home Win</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>77.00%</t>
+          <t>76.00%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1794,27 +1789,27 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>OOUUUU</t>
+          <t>DWDWWW</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>UUOUUU</t>
+          <t>LDLLLL</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Atl. Tucuman averages 1.0 goals at home. Ind. Rivadavia averages 1.4 goals at away. Atl. Tucuman concedes 0.8 goals at home. Ind. Rivadavia concedes 0.7 goals at away. Both sides look capable of goals.</t>
+          <t>GAIS has won 4 of their last 6 home games. Halmstad has won 0 of their last 6 home games. Halmstad concedes 2.5 goals at away. Strong home record supports this.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16M 3W 5D 8L 15-20 (0.9-1.2) | Home: 8M 2W 5D 1L 8-6 (1.0-0.8)</t>
+          <t>14M 5W 4D 5L 18-14 (1.3-1.0) | Home: 7M 4W 2D 1L 11-2 (1.6-0.3)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>17M 10W 4D 3L 30-17 (1.8-1.0) | Away: 7M 4W 3D 0L 10-5 (1.4-0.7)</t>
+          <t>13M 1W 3D 9L 10-28 (0.8-2.2) | Away: 6M 0W 1D 5L 4-15 (0.7-2.5)</t>
         </is>
       </c>
       <c r="O18" t="b">
@@ -1834,62 +1829,62 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Home Win</t>
+          <t>Away Win</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>77.00%</t>
+          <t>76.00%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>LLWWLW</t>
+          <t>LDDWDD</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>WDLLLL</t>
+          <t>WWWWLW</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Brann has won 3 of their last 6 home games. Valerenga has won 1 of their last 6 home games. Valerenga concedes 2.2 goals at away. Strong home record supports this.</t>
+          <t>Viking has won 5 of their last 6 home games. Aalesund has won 1 of their last 6 home games. Aalesund concedes 2.0 goals at home. Away form makes them favourites.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O19" t="b">
@@ -1899,7 +1894,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SE Allsvenskan</t>
+          <t>BR Serie A</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1909,62 +1904,62 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>15:30:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Halmstad</t>
+          <t>Botafogo RJ</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Home Win</t>
+          <t>Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>76.00%</t>
+          <t>71.00%</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DWDWWW</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>LDLLLL</t>
+          <t>OOOUUO</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>GAIS has won 4 of their last 6 home games. Halmstad has won 0 of their last 6 home games. Halmstad concedes 2.5 goals at away. Strong home record supports this.</t>
+          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. Botafogo RJ concedes 1.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>14M 5W 4D 5L 18-14 (1.3-1.0) | Home: 7M 4W 2D 1L 11-2 (1.6-0.3)</t>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>13M 1W 3D 9L 10-28 (0.8-2.2) | Away: 6M 0W 1D 5L 4-15 (0.7-2.5)</t>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
         </is>
       </c>
       <c r="O20" t="b">
@@ -1984,22 +1979,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>22:30:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Flamengo RJ</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sao Paulo</t>
+          <t>Botafogo RJ</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Both Teams to Score</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2009,37 +2004,37 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>76.00%</t>
+          <t>71.00%</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>OOUOOO</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>UUOOOU</t>
+          <t>OOOUUO</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Flamengo RJ averages 2.0 goals at home. Sao Paulo averages 0.9 goals at away. Flamengo RJ concedes 0.9 goals at home. Sao Paulo concedes 1.4 goals at away. Both sides look capable of goals.</t>
+          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Both teams tend to concede (Cruzeiro concedes 1.2 goals at home., Botafogo RJ concedes 1.9 goals at away.), making goals at both ends likely.</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>18M 11W 4D 3L 35.0-16.0 (1.9-0.9) | Home: 8M 5W 2D 1L 16.0-7.0 (2.0-0.9)</t>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>19M 7W 4D 8L 24.0-22.0 (1.3-1.2) | Away: 10M 2W 2D 6L 9.0-14.0 (0.9-1.4)</t>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
         </is>
       </c>
       <c r="O21" t="b">
@@ -2049,7 +2044,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>BR Serie A</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2059,62 +2054,62 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>18:15:00</t>
+          <t>22:30:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Flamengo RJ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Sao Paulo</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Away Win</t>
+          <t>Home Win</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>76.00%</t>
+          <t>68.00%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>LDDWDD</t>
+          <t>WWWDLW</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>WWWWLW</t>
+          <t>DLLLLL</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Viking has won 5 of their last 6 home games. Aalesund has won 1 of their last 6 home games. Aalesund concedes 2.0 goals at home. Away form makes them favourites.</t>
+          <t>Flamengo RJ has won 4 of their last 6 home games. Sao Paulo has won 0 of their last 6 home games. Sao Paulo concedes 1.4 goals at away. Strong home record supports this.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
+          <t>18M 11W 4D 3L 35.0-16.0 (1.9-0.9) | Home: 8M 5W 2D 1L 16.0-7.0 (2.0-0.9)</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
+          <t>19M 7W 4D 8L 24.0-22.0 (1.3-1.2) | Away: 10M 2W 2D 6L 9.0-14.0 (0.9-1.4)</t>
         </is>
       </c>
       <c r="O22" t="b">
@@ -2124,7 +2119,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2134,22 +2129,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>22:30:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bragantino</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Both Teams to Score</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2159,7 +2154,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>68.00%</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2169,37 +2164,37 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>OOOUUO</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>UOUOOO</t>
+          <t>UOUOUO</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Bragantino averages 1.8 goals at home. Coritiba averages 1.4 goals at away. Bragantino concedes 1.0 goals at home. Coritiba concedes 1.6 goals at away. Both sides look capable of goals.</t>
+          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Both teams tend to concede (Aalesund concedes 2.0 goals at home., Viking concedes 0.9 goals at away.), making goals at both ends likely.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>19M 9W 3D 7L 26.0-20.0 (1.4-1.1) | Home: 9M 5W 1D 3L 16.0-9.0 (1.8-1.0)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>19M 7W 5D 7L 25.0-27.0 (1.3-1.4) | Away: 10M 4W 2D 4L 14.0-16.0 (1.4-1.6)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PL Ekstraklasa</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2209,22 +2204,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16:30:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Both Teams to Score</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2234,37 +2229,37 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>73.00%</t>
+          <t>67.00%</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>OUUUOO</t>
+          <t>OUOOOO</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>OUOUOO</t>
+          <t>UUOUUO</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Widzew Lodz averages 1.4 goals at home. Motor Lublin averages 1.4 goals at away. Widzew Lodz concedes 0.9 goals at home. Motor Lublin concedes 1.9 goals at away. Both sides look capable of goals.</t>
+          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Both teams tend to concede (Brann concedes 1.3 goals at home., Valerenga concedes 2.2 goals at away.), making goals at both ends likely.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>34M 12W 6D 16L 41-41 (1.2-1.2) | Home: 17M 9W 4D 4L 24-16 (1.4-0.9)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>34M 10W 13D 11L 46-53 (1.4-1.6) | Away: 17M 5W 4D 8L 23-33 (1.4-1.9)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O24" t="b">
@@ -2274,7 +2269,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>CH Super League</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2284,22 +2279,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>22:30:00</t>
+          <t>15:30:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gremio</t>
+          <t>St. Gallen</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2309,37 +2304,37 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>72.00%</t>
+          <t>67.00%</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>6/10</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UUUUOO</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>OUOUUU</t>
+          <t>OOOOOU</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Gremio averages 1.7 goals at home. Fluminense averages 1.2 goals at away. Gremio concedes 1.2 goals at home. Fluminense concedes 1.4 goals at away. Both sides look capable of goals.</t>
+          <t>St. Gallen averages 1.7 goals at home. Zurich concedes 1.9 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>19M 5W 6D 8L 21.0-25.0 (1.1-1.3) | Home: 9M 5W 2D 2L 15.0-11.0 (1.7-1.2)</t>
+          <t>38M 20W 10D 8L 72-47 (1.9-1.2) | Home: 19M 10W 3D 6L 33-23 (1.7-1.2)</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>19M 9W 5D 5L 29.0-24.0 (1.5-1.3) | Away: 9M 2W 3D 4L 11.0-13.0 (1.2-1.4)</t>
+          <t>38M 11W 5D 22L 49-72 (1.3-1.9) | Away: 19M 4W 4D 11L 20-36 (1.1-1.9)</t>
         </is>
       </c>
       <c r="O25" t="b">
@@ -2349,7 +2344,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>DK Superliga</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2359,17 +2354,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>20:00:00</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Botafogo RJ</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2384,37 +2379,32 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>71.00%</t>
+          <t>66.00%</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>OOUOOU</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>OOOUUO</t>
+          <t>OOOOOO</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. Botafogo RJ concedes 1.9 goals at away. Both sides look capable of goals.</t>
+          <t>FC Copenhagen averages 2.1 goals at home. Lyngby averages 0.0 goals at away. FC Copenhagen concedes 1.2 goals at home. Lyngby concedes 0.0 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
+          <t>32M 15W 6D 11L 67-44 (2.1-1.4) | Home: 16M 7W 4D 5L 33-19 (2.1-1.2)</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
+          <t>0M 0W 0D 0L 0-0 (0.0-0.0)</t>
         </is>
       </c>
       <c r="O26" t="b">
@@ -2424,7 +2414,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>CH Super League</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2434,17 +2424,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>20:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Young Boys</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Botafogo RJ</t>
+          <t>Sion</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2459,37 +2449,37 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>71.00%</t>
+          <t>66.00%</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>OOUOOU</t>
+          <t>OUUOOO</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>OOOUUO</t>
+          <t>OOOUOO</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Both teams tend to concede (Cruzeiro concedes 1.2 goals at home., Botafogo RJ concedes 1.9 goals at away.), making goals at both ends likely.</t>
+          <t>Young Boys averages 2.3 goals at home. Sion averages 1.8 goals at away. Both teams tend to concede (Young Boys concedes 1.3 goals at home., Sion concedes 1.4 goals at away.), making goals at both ends likely.</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
+          <t>38M 15W 10D 13L 80-69 (2.1-1.8) | Home: 19M 9W 5D 5L 43-25 (2.3-1.3)</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
+          <t>38M 16W 15D 7L 63-40 (1.7-1.1) | Away: 19M 7W 8D 4L 34-26 (1.8-1.4)</t>
         </is>
       </c>
       <c r="O27" t="b">
@@ -2499,7 +2489,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SE Allsvenskan</t>
+          <t>DK Superliga</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2509,22 +2499,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>15:30:00</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Halmstad</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Both Teams to Score</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2534,37 +2524,32 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>70.00%</t>
+          <t>65.00%</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>UOUUOU</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>OUUUOO</t>
+          <t>OOOOOO</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>GAIS averages 1.6 goals at home. Halmstad averages 0.7 goals at away. GAIS concedes 0.3 goals at home. Halmstad concedes 2.5 goals at away. Both sides look capable of goals.</t>
+          <t>FC Copenhagen averages 2.1 goals at home. Lyngby averages 0.0 goals at away. Both teams tend to concede (FC Copenhagen concedes 1.2 goals at home., Lyngby concedes 0.0 goals at away.), making goals at both ends likely.</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>14M 5W 4D 5L 18-14 (1.3-1.0) | Home: 7M 4W 2D 1L 11-2 (1.6-0.3)</t>
+          <t>32M 15W 6D 11L 67-44 (2.1-1.4) | Home: 16M 7W 4D 5L 33-19 (2.1-1.2)</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>13M 1W 3D 9L 10-28 (0.8-2.2) | Away: 6M 0W 1D 5L 4-15 (0.7-2.5)</t>
+          <t>0M 0W 0D 0L 0-0 (0.0-0.0)</t>
         </is>
       </c>
       <c r="O28" t="b">
@@ -2574,7 +2559,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2584,22 +2569,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>23:30:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Atletico-MG</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Over 3.5 Goals</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2609,37 +2594,37 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>69.00%</t>
+          <t>64.00%</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>OOUUUU</t>
+          <t>OUOOOO</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>OUUOUU</t>
+          <t>UUOUUO</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Palmeiras averages 1.8 goals at home. Atletico-MG averages 0.9 goals at away. Palmeiras concedes 0.7 goals at home. Atletico-MG concedes 1.1 goals at away. Both sides look capable of goals.</t>
+          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Brann concedes 1.3 goals at home. Valerenga concedes 2.2 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>19M 13W 5D 1L 33.0-14.0 (1.7-0.7) | Home: 9M 7W 2D 0L 16.0-6.0 (1.8-0.7)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>19M 7W 4D 8L 23.0-24.0 (1.2-1.3) | Away: 10M 3W 0D 7L 9.0-11.0 (0.9-1.1)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O29" t="b">
@@ -2649,7 +2634,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BR Serie A</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2659,62 +2644,62 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>22:30:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Flamengo RJ</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sao Paulo</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Home Win</t>
+          <t>Over 3.5 Goals</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>68.00%</t>
+          <t>64.00%</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>WWWDLW</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>DLLLLL</t>
+          <t>UOUOUO</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Flamengo RJ has won 4 of their last 6 home games. Sao Paulo has won 0 of their last 6 home games. Sao Paulo concedes 1.4 goals at away. Strong home record supports this.</t>
+          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. Viking concedes 0.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>18M 11W 4D 3L 35.0-16.0 (1.9-0.9) | Home: 8M 5W 2D 1L 16.0-7.0 (2.0-0.9)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>19M 7W 4D 8L 24.0-22.0 (1.3-1.2) | Away: 10M 2W 2D 6L 9.0-14.0 (0.9-1.4)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O30" t="b">
@@ -2724,7 +2709,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>CH Super League</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2734,22 +2719,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>KFUM Oslo</t>
+          <t>Young Boys</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Molde</t>
+          <t>Sion</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2759,37 +2744,37 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>68.00%</t>
+          <t>63.00%</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>OUUUUU</t>
+          <t>OUUOOO</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>OUUUOO</t>
+          <t>OOOUOO</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>KFUM Oslo averages 0.9 goals at home. Molde averages 1.0 goals at away. KFUM Oslo concedes 0.9 goals at home. Molde concedes 1.8 goals at away. Both sides look capable of goals.</t>
+          <t>Young Boys averages 2.3 goals at home. Sion averages 1.8 goals at away. Young Boys concedes 1.3 goals at home. Sion concedes 1.4 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>13M 3W 3D 7L 13-21 (1.0-1.6) | Home: 7M 3W 1D 3L 6-6 (0.9-0.9)</t>
+          <t>38M 15W 10D 13L 80-69 (2.1-1.8) | Home: 19M 9W 5D 5L 43-25 (2.3-1.3)</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>13M 6W 2D 5L 21-17 (1.6-1.3) | Away: 6M 1W 2D 3L 6-11 (1.0-1.8)</t>
+          <t>38M 16W 15D 7L 63-40 (1.7-1.1) | Away: 19M 7W 8D 4L 34-26 (1.8-1.4)</t>
         </is>
       </c>
       <c r="O31" t="b">
@@ -2809,22 +2794,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>18:15:00</t>
+          <t>13:30:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Both Teams to Score</t>
+          <t>Home team Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2834,37 +2819,37 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>68.00%</t>
+          <t>63.00%</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>OOUOOO</t>
+          <t>OUOOOO</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>UOUOUO</t>
+          <t>UUOUUO</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Both teams tend to concede (Aalesund concedes 2.0 goals at home., Viking concedes 0.9 goals at away.), making goals at both ends likely.</t>
+          <t>Brann averages 1.5 goals at home. Valerenga concedes 2.2 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
+          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
+          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
         </is>
       </c>
       <c r="O32" t="b">
@@ -2874,7 +2859,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>FI Veikkausliiga</t>
+          <t>NO Eliteserien</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2884,22 +2869,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>18:15:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Viking</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Away team Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2909,37 +2894,37 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>67.00%</t>
+          <t>62.00%</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>UUUOUU</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>UUOUUU</t>
+          <t>UOUOUO</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Inter Turku averages 1.1 goals at home. Gnistan averages 1.0 goals at away. Inter Turku concedes 0.5 goals at home. Gnistan concedes 0.9 goals at away. Both sides look capable of goals.</t>
+          <t>Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. The away side’s attack looks likely to score well.</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>16M 8W 7D 1L 23-12 (1.4-0.8) | Home: 8M 4W 4D 0L 9-4 (1.1-0.5)</t>
+          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>16M 7W 4D 5L 25-20 (1.6-1.2) | Away: 8M 2W 3D 3L 8-7 (1.0-0.9)</t>
+          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
         </is>
       </c>
       <c r="O33" t="b">
@@ -2949,7 +2934,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>DK Superliga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2959,22 +2944,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Both Teams to Score</t>
+          <t>Home team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2984,37 +2969,32 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>67.00%</t>
+          <t>61.00%</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>OUOOOO</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>UUOUUO</t>
+          <t>OOOOOO</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Both teams tend to concede (Brann concedes 1.3 goals at home., Valerenga concedes 2.2 goals at away.), making goals at both ends likely.</t>
+          <t>FC Copenhagen averages 2.1 goals at home. Lyngby concedes 0.0 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
+          <t>32M 15W 6D 11L 67-44 (2.1-1.4) | Home: 16M 7W 4D 5L 33-19 (2.1-1.2)</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
+          <t>0M 0W 0D 0L 0-0 (0.0-0.0)</t>
         </is>
       </c>
       <c r="O34" t="b">
@@ -3024,7 +3004,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CH Super League</t>
+          <t>BR Serie A</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3034,17 +3014,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>15:30:00</t>
+          <t>22:30:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>St. Gallen</t>
+          <t>Flamengo RJ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Sao Paulo</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3059,37 +3039,37 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>67.00%</t>
+          <t>61.00%</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>6/10</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>OOUOOU</t>
+          <t>OOUOOO</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>OOOOOU</t>
+          <t>UUOOOU</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>St. Gallen averages 1.7 goals at home. Zurich concedes 1.9 goals at away. The home side’s attack should produce the required goals.</t>
+          <t>Flamengo RJ averages 2.0 goals at home. Sao Paulo concedes 1.4 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>38M 20W 10D 8L 72-47 (1.9-1.2) | Home: 19M 10W 3D 6L 33-23 (1.7-1.2)</t>
+          <t>18M 11W 4D 3L 35.0-16.0 (1.9-0.9) | Home: 8M 5W 2D 1L 16.0-7.0 (2.0-0.9)</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>38M 11W 5D 22L 49-72 (1.3-1.9) | Away: 19M 4W 4D 11L 20-36 (1.1-1.9)</t>
+          <t>19M 7W 4D 8L 24.0-22.0 (1.3-1.2) | Away: 10M 2W 2D 6L 9.0-14.0 (0.9-1.4)</t>
         </is>
       </c>
       <c r="O35" t="b">
@@ -3099,7 +3079,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AR Liga Profesional</t>
+          <t>CH Super League</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3109,22 +3089,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>21:15:00</t>
+          <t>15:30:00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Estudiantes L.P.</t>
+          <t>St. Gallen</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Independiente</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Over 2.5 Goals</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3134,37 +3114,37 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>67.00%</t>
+          <t>61.00%</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>7/10</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>UUOOUU</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>UOUUOO</t>
+          <t>OOOOOU</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Estudiantes L.P. averages 1.4 goals at home. Independiente averages 1.1 goals at away. Estudiantes L.P. concedes 0.5 goals at home. Independiente concedes 1.6 goals at away. Both sides look capable of goals.</t>
+          <t>St. Gallen averages 1.7 goals at home. Zurich averages 1.1 goals at away. St. Gallen concedes 1.2 goals at home. Zurich concedes 1.9 goals at away. Both sides look capable of goals.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>16M 9W 4D 3L 19-7 (1.2-0.4) | Home: 8M 5W 1D 2L 11-4 (1.4-0.5)</t>
+          <t>38M 20W 10D 8L 72-47 (1.9-1.2) | Home: 19M 10W 3D 6L 33-23 (1.7-1.2)</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>17M 6W 6D 5L 25-23 (1.5-1.4) | Away: 9M 2W 3D 4L 10-14 (1.1-1.6)</t>
+          <t>38M 11W 5D 22L 49-72 (1.3-1.9) | Away: 19M 4W 4D 11L 20-36 (1.1-1.9)</t>
         </is>
       </c>
       <c r="O36" t="b">
@@ -3174,7 +3154,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CH Super League</t>
+          <t>SE Allsvenskan</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3184,22 +3164,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>15:30:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Young Boys</t>
+          <t>GAIS</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sion</t>
+          <t>Halmstad</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Both Teams to Score</t>
+          <t>Home team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3209,37 +3189,37 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>66.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>7/8</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>OUUOOO</t>
+          <t>UOUUOU</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>OOOUOO</t>
+          <t>OUUUOO</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Young Boys averages 2.3 goals at home. Sion averages 1.8 goals at away. Both teams tend to concede (Young Boys concedes 1.3 goals at home., Sion concedes 1.4 goals at away.), making goals at both ends likely.</t>
+          <t>GAIS averages 1.6 goals at home. Halmstad concedes 2.5 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>38M 15W 10D 13L 80-69 (2.1-1.8) | Home: 19M 9W 5D 5L 43-25 (2.3-1.3)</t>
+          <t>14M 5W 4D 5L 18-14 (1.3-1.0) | Home: 7M 4W 2D 1L 11-2 (1.6-0.3)</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>38M 16W 15D 7L 63-40 (1.7-1.1) | Away: 19M 7W 8D 4L 34-26 (1.8-1.4)</t>
+          <t>13M 1W 3D 9L 10-28 (0.8-2.2) | Away: 6M 0W 1D 5L 4-15 (0.7-2.5)</t>
         </is>
       </c>
       <c r="O37" t="b">
@@ -3249,7 +3229,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PL Ekstraklasa</t>
+          <t>BR Serie A</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3259,22 +3239,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>13:45:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Rakow</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Botafogo RJ</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Home team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3284,37 +3264,37 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>65.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>UUOUUO</t>
+          <t>OOUOOU</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>OOUOOO</t>
+          <t>OOOUUO</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Rakow averages 1.4 goals at home. Wisla Plock averages 1.1 goals at away. Rakow concedes 0.9 goals at home. Wisla Plock concedes 1.3 goals at away. Both sides look capable of goals.</t>
+          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ concedes 1.9 goals at away. The home side’s attack should produce the required goals.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>34M 16W 7D 11L 51-40 (1.5-1.2) | Home: 17M 8W 4D 5L 23-15 (1.4-0.9)</t>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>34M 12W 10D 12L 34-38 (1.0-1.1) | Away: 17M 4W 7D 6L 18-22 (1.1-1.3)</t>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
         </is>
       </c>
       <c r="O38" t="b">
@@ -3324,7 +3304,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>DK Superliga</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3334,22 +3314,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Sonderjyske</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bodo/Glimt</t>
+          <t>Midtjylland</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Over 1.5 Goals</t>
+          <t>Away team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3359,47 +3339,47 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>64.00%</t>
+          <t>59.00%</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>UUUUUO</t>
+          <t>UUUOOO</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>OUUOOU</t>
+          <t>OUOOUU</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Sandefjord averages 1.0 goals at home. Bodo/Glimt averages 2.0 goals at away. Sandefjord concedes 0.8 goals at home. Bodo/Glimt concedes 1.3 goals at away. Both sides look capable of goals.</t>
+          <t>Midtjylland averages 1.8 goals at away. Sonderjyske concedes 1.2 goals at home. The away side’s attack looks likely to score well.</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>13M 4W 3D 6L 13-17 (1.0-1.3) | Home: 6M 2W 3D 1L 6-5 (1.0-0.8)</t>
+          <t>32M 12W 8D 12L 44-49 (1.4-1.5) | Home: 16M 8W 3D 5L 25-20 (1.6-1.2)</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>14M 10W 2D 2L 34-11 (2.4-0.8) | Away: 7M 4W 2D 1L 14-9 (2.0-1.3)</t>
+          <t>32M 16W 12D 4L 72-36 (2.2-1.1) | Away: 16M 8W 6D 2L 29-12 (1.8-0.8)</t>
         </is>
       </c>
       <c r="O39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NO Eliteserien</t>
+          <t>SE Allsvenskan</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3409,22 +3389,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Brommapojkarna</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Hammarby</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Over 3.5 Goals</t>
+          <t>Away team Over 1.5 Goals</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3434,7 +3414,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>64.00%</t>
+          <t>58.00%</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3444,27 +3424,27 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>OUOOOO</t>
+          <t>-OOUUO</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>UUOUUO</t>
+          <t>UUUUOO</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Brann averages 1.5 goals at home. Valerenga averages 0.7 goals at away. Brann concedes 1.3 goals at home. Valerenga concedes 2.2 goals at away. Both sides look capable of goals.</t>
+          <t>Hammarby averages 1.0 goals at away. Brommapojkarna concedes 1.4 goals at home. The away side’s attack looks likely to score well.</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>14M 6W 1D 7L 28-22 (2.0-1.6) | Home: 6M 3W 0D 3L 9-8 (1.5-1.3)</t>
+          <t>13M 4W 4D 5L 18-21 (1.4-1.6) | Home: 5M 1W 2D 2L 6-7 (1.2-1.4)</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>13M 5W 2D 6L 19-22 (1.5-1.7) | Away: 6M 1W 1D 4L 4-13 (0.7-2.2)</t>
+          <t>14M 8W 2D 4L 32-14 (2.3-1.0) | Away: 6M 2W 1D 3L 6-9 (1.0-1.5)</t>
         </is>
       </c>
       <c r="O40" t="b">
@@ -3474,75 +3454,520 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>SE Allsvenskan</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Malmo FF</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Elfsborg</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Home team Over 1.5 Goals</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>58.00%</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>OOOOOO</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>OUOUOU</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Malmo FF averages 3.0 goals at home. Elfsborg concedes 1.3 goals at away. The home side’s attack should produce the required goals.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>13M 6W 2D 5L 27-22 (2.1-1.7) | Home: 6M 3W 0D 3L 18-12 (3.0-2.0)</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>14M 4W 6D 4L 18-17 (1.3-1.2) | Away: 6M 1W 3D 2L 7-8 (1.2-1.3)</t>
+        </is>
+      </c>
+      <c r="O41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>NO Eliteserien</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>26-07-2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>18:15:00</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Aalesund</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Viking</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>16:00:00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Sarpsborg 08</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>HamKam</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Home team Over 1.5 Goals</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>56.00%</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>UUUOOU</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>OUOOOO</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Sarpsborg 08 averages 1.2 goals at home. HamKam concedes 2.3 goals at away. The home side’s attack should produce the required goals.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>13M 5W 3D 5L 14-16 (1.1-1.2) | Home: 6M 3W 2D 1L 7-5 (1.2-0.8)</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>13M 5W 3D 5L 20-25 (1.5-1.9) | Away: 6M 0W 3D 3L 7-14 (1.2-2.3)</t>
+        </is>
+      </c>
+      <c r="O42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BR Serie A</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>20:00:00</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Botafogo RJ</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
         <is>
           <t>Over 3.5 Goals</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>64.00%</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>OOUOOU</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>OOOUUO</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Cruzeiro averages 1.6 goals at home. Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. Botafogo RJ concedes 1.9 goals at away. Both sides look capable of goals.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
+        </is>
+      </c>
+      <c r="O43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BR Serie A</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>20:00:00</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Botafogo RJ</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Away team Over 1.5 Goals</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>49.00%</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>OOUOOU</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>OOOUUO</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Botafogo RJ averages 1.6 goals at away. Cruzeiro concedes 1.2 goals at home. The away side’s attack looks likely to score well.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>19M 7W 6D 6L 26.0-29.0 (1.4-1.5) | Home: 10M 4W 4D 2L 16.0-12.0 (1.6-1.2)</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>19M 7W 5D 7L 33.0-32.0 (1.7-1.7) | Away: 10M 3W 2D 5L 16.0-19.0 (1.6-1.9)</t>
+        </is>
+      </c>
+      <c r="O44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AR Liga Profesional</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>19:00:00</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Atl. Tucuman</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Ind. Rivadavia</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Away team Over 1.5 Goals</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>48.00%</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>OOUOOO</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>UOUOUO</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Aalesund averages 1.7 goals at home. Viking averages 1.4 goals at away. Aalesund concedes 2.0 goals at home. Viking concedes 0.9 goals at away. Both sides look capable of goals.</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>13M 2W 6D 5L 18-28 (1.4-2.2) | Home: 7M 1W 4D 2L 12-14 (1.7-2.0)</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>13M 11W 0D 2L 33-13 (2.5-1.0) | Away: 7M 5W 0D 2L 10-6 (1.4-0.9)</t>
-        </is>
-      </c>
-      <c r="O41" t="b">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>OOUUUU</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>UUOUUU</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Ind. Rivadavia averages 1.4 goals at away. Atl. Tucuman concedes 0.8 goals at home. The away side’s attack looks likely to score well.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>16M 3W 5D 8L 15-20 (0.9-1.2) | Home: 8M 2W 5D 1L 8-6 (1.0-0.8)</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>17M 10W 4D 3L 30-17 (1.8-1.0) | Away: 7M 4W 3D 0L 10-5 (1.4-0.7)</t>
+        </is>
+      </c>
+      <c r="O45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DK Superliga</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FC Copenhagen</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Over 3.5 Goals</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>45.00%</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>OOOOOO</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>FC Copenhagen averages 2.1 goals at home. Lyngby averages 0.0 goals at away. FC Copenhagen concedes 1.2 goals at home. Lyngby concedes 0.0 goals at away. Both sides look capable of goals.</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>32M 15W 6D 11L 67-44 (2.1-1.4) | Home: 16M 7W 4D 5L 33-19 (2.1-1.2)</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0M 0W 0D 0L 0-0 (0.0-0.0)</t>
+        </is>
+      </c>
+      <c r="O46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CH Super League</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>St. Gallen</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Home team Over 2.5 Goals</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>40.00%</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>OOUOOU</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>OOOOOU</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>St. Gallen averages 1.7 goals at home. Zurich concedes 1.9 goals at away. The home side’s attack should produce the required goals.</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>38M 20W 10D 8L 72-47 (1.9-1.2) | Home: 19M 10W 3D 6L 33-23 (1.7-1.2)</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>38M 11W 5D 22L 49-72 (1.3-1.9) | Away: 19M 4W 4D 11L 20-36 (1.1-1.9)</t>
+        </is>
+      </c>
+      <c r="O47" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>